<commit_message>
added and fixed some features
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Kerjaan\GIS Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29F7144-8D21-477A-82DC-612E77DDC943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{610F79C2-B48E-4738-812A-C1C31CF65F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="196">
   <si>
     <t>Client</t>
   </si>
@@ -144,9 +144,6 @@
     <t>Prima Cahaya Timur</t>
   </si>
   <si>
-    <t>Wooden</t>
-  </si>
-  <si>
     <t>Royal Sentra Energi</t>
   </si>
   <si>
@@ -426,9 +423,6 @@
     <t>Kalimantan Timur</t>
   </si>
   <si>
-    <t>Balikpapan</t>
-  </si>
-  <si>
     <t>Buana Karya Samudera</t>
   </si>
   <si>
@@ -622,6 +616,9 @@
   </si>
   <si>
     <t>Kota Surabaya</t>
+  </si>
+  <si>
+    <t>Kota Balikpapan</t>
   </si>
 </sst>
 </file>
@@ -946,10 +943,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -1067,7 +1064,7 @@
         <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1081,7 +1078,7 @@
         <v>18</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1232,7 +1229,7 @@
         <v>10</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>4</v>
@@ -1263,7 +1260,7 @@
         <v>36</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1274,7 +1271,7 @@
         <v>10</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>4</v>
@@ -1288,10 +1285,10 @@
         <v>10</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1302,7 +1299,7 @@
         <v>10</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>31</v>
@@ -1319,7 +1316,7 @@
         <v>7</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1330,10 +1327,10 @@
         <v>10</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1344,10 +1341,10 @@
         <v>10</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1358,10 +1355,10 @@
         <v>10</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1372,10 +1369,10 @@
         <v>10</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1386,10 +1383,10 @@
         <v>10</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1400,7 +1397,7 @@
         <v>10</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>25</v>
@@ -1414,10 +1411,10 @@
         <v>10</v>
       </c>
       <c r="C34" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -1428,63 +1425,63 @@
         <v>10</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="C36" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="D36" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C38" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C39" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>31</v>
@@ -1492,10 +1489,10 @@
     </row>
     <row r="40" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>58</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>5</v>
@@ -1506,27 +1503,27 @@
     </row>
     <row r="41" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C41" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C42" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>4</v>
@@ -1534,97 +1531,97 @@
     </row>
     <row r="43" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C44" s="4" t="s">
+      <c r="D44" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>81</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1632,13 +1629,13 @@
     </row>
     <row r="50" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>31</v>
@@ -1646,41 +1643,41 @@
     </row>
     <row r="51" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C51" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D51" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>4</v>
@@ -1688,69 +1685,69 @@
     </row>
     <row r="54" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C56" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D56" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>33</v>
@@ -1758,13 +1755,13 @@
     </row>
     <row r="59" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>31</v>
@@ -1772,10 +1769,10 @@
     </row>
     <row r="60" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>13</v>
@@ -1786,10 +1783,10 @@
     </row>
     <row r="61" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>5</v>
@@ -1800,41 +1797,41 @@
     </row>
     <row r="62" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>31</v>
@@ -1842,41 +1839,41 @@
     </row>
     <row r="65" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C65" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D65" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>31</v>
@@ -1884,13 +1881,13 @@
     </row>
     <row r="68" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>31</v>
@@ -1898,38 +1895,38 @@
     </row>
     <row r="69" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>7</v>
@@ -1940,195 +1937,195 @@
     </row>
     <row r="72" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B72" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B72" s="4" t="s">
+      <c r="C72" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="D72" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B73" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="C73" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C73" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="D73" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B74" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B74" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B75" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B75" s="4" t="s">
-        <v>107</v>
-      </c>
       <c r="C75" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D78" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B80" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>116</v>
-      </c>
       <c r="D80" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C83" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C84" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D84" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="D84" s="5" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>33</v>
@@ -2136,13 +2133,13 @@
     </row>
     <row r="86" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>4</v>
@@ -2150,181 +2147,181 @@
     </row>
     <row r="87" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C92" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D92" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="D92" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C95" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C96" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B96" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="C96" s="7" t="s">
+      <c r="D96" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="D96" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C97" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B97" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C97" s="7" t="s">
+      <c r="D97" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="D97" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C98" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B98" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C98" s="7" t="s">
+      <c r="D98" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="D98" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>4</v>
@@ -2332,55 +2329,55 @@
     </row>
     <row r="100" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C101" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B101" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="C101" s="7" t="s">
-        <v>132</v>
-      </c>
       <c r="D101" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B102" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C102" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C102" s="7" t="s">
-        <v>133</v>
-      </c>
       <c r="D102" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>131</v>
+        <v>195</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>4</v>
@@ -2388,13 +2385,13 @@
     </row>
     <row r="104" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>4</v>
@@ -2402,13 +2399,13 @@
     </row>
     <row r="105" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>4</v>
@@ -2416,13 +2413,13 @@
     </row>
     <row r="106" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>4</v>
@@ -2430,27 +2427,27 @@
     </row>
     <row r="107" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B107" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C107" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="C107" s="7" t="s">
-        <v>140</v>
-      </c>
       <c r="D107" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>4</v>
@@ -2458,27 +2455,27 @@
     </row>
     <row r="109" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B109" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D109" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>4</v>
@@ -2486,27 +2483,27 @@
     </row>
     <row r="111" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C111" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D111" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="B111" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="C111" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B112" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C112" s="7" t="s">
         <v>144</v>
-      </c>
-      <c r="C112" s="7" t="s">
-        <v>146</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2514,13 +2511,13 @@
     </row>
     <row r="113" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B113" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2528,10 +2525,10 @@
     </row>
     <row r="114" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C114" s="7" t="s">
         <v>34</v>
@@ -2542,83 +2539,83 @@
     </row>
     <row r="115" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D115" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C116" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D119" s="5" t="s">
         <v>150</v>
-      </c>
-      <c r="B119" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="C119" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>4</v>
@@ -2626,27 +2623,27 @@
     </row>
     <row r="121" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B121" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>4</v>
@@ -2654,69 +2651,69 @@
     </row>
     <row r="123" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C123" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D123" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="C124" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B124" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C124" s="7" t="s">
-        <v>158</v>
-      </c>
       <c r="D124" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B125" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C125" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B125" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C125" s="7" t="s">
-        <v>161</v>
-      </c>
       <c r="D125" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B126" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C126" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C127" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>4</v>
@@ -2724,13 +2721,13 @@
     </row>
     <row r="128" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C128" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>4</v>
@@ -2738,41 +2735,41 @@
     </row>
     <row r="129" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B129" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D129" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="B129" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="C129" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C130" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B131" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C131" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>4</v>
@@ -2780,41 +2777,41 @@
     </row>
     <row r="132" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B132" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C132" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B133" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C133" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C134" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>4</v>
@@ -2822,41 +2819,41 @@
     </row>
     <row r="135" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C135" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B136" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B136" s="7" t="s">
-        <v>171</v>
-      </c>
       <c r="C136" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B137" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C137" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>4</v>
@@ -2864,27 +2861,27 @@
     </row>
     <row r="138" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C138" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B139" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C139" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>4</v>
@@ -2892,44 +2889,44 @@
     </row>
     <row r="140" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B140" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C140" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C141" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B141" s="7" t="s">
+      <c r="D141" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="C141" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B142" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="C142" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D142" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="B142" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="C142" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v1.0.5 export system stabilization and UI enhancement
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Kerjaan\GIS Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{610F79C2-B48E-4738-812A-C1C31CF65F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77377A36-BD65-457B-AAE2-5DA786D80DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -459,9 +459,6 @@
     <t>Kepulauan Riau</t>
   </si>
   <si>
-    <t>Batam</t>
-  </si>
-  <si>
     <t>Pipe</t>
   </si>
   <si>
@@ -516,9 +513,6 @@
     <t>Riau</t>
   </si>
   <si>
-    <t>Dumai</t>
-  </si>
-  <si>
     <t>Cargo</t>
   </si>
   <si>
@@ -619,6 +613,12 @@
   </si>
   <si>
     <t>Kota Balikpapan</t>
+  </si>
+  <si>
+    <t>Kota Batam</t>
+  </si>
+  <si>
+    <t>Kota Dumai</t>
   </si>
 </sst>
 </file>
@@ -943,10 +943,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1078,7 +1078,7 @@
         <v>18</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1229,7 +1229,7 @@
         <v>10</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>4</v>
@@ -1548,7 +1548,7 @@
         <v>74</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>75</v>
@@ -1562,7 +1562,7 @@
         <v>74</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>37</v>
@@ -1576,7 +1576,7 @@
         <v>74</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>37</v>
@@ -1590,7 +1590,7 @@
         <v>74</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>77</v>
@@ -1618,7 +1618,7 @@
         <v>79</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>80</v>
@@ -1632,7 +1632,7 @@
         <v>79</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>81</v>
@@ -1646,7 +1646,7 @@
         <v>79</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>84</v>
@@ -1660,7 +1660,7 @@
         <v>79</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>84</v>
@@ -1674,10 +1674,10 @@
         <v>79</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>4</v>
@@ -1688,7 +1688,7 @@
         <v>79</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>66</v>
@@ -1702,7 +1702,7 @@
         <v>79</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>88</v>
@@ -1716,7 +1716,7 @@
         <v>79</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>89</v>
@@ -1730,7 +1730,7 @@
         <v>79</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>91</v>
@@ -1744,7 +1744,7 @@
         <v>79</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>92</v>
@@ -1758,7 +1758,7 @@
         <v>79</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>93</v>
@@ -1772,7 +1772,7 @@
         <v>79</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>13</v>
@@ -1786,7 +1786,7 @@
         <v>79</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>5</v>
@@ -1800,7 +1800,7 @@
         <v>79</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>5</v>
@@ -1814,7 +1814,7 @@
         <v>79</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -1828,7 +1828,7 @@
         <v>79</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>95</v>
@@ -1842,7 +1842,7 @@
         <v>79</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>96</v>
@@ -1856,7 +1856,7 @@
         <v>79</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>98</v>
@@ -1870,7 +1870,7 @@
         <v>79</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>99</v>
@@ -1884,7 +1884,7 @@
         <v>79</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>100</v>
@@ -1898,7 +1898,7 @@
         <v>79</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>7</v>
@@ -1912,7 +1912,7 @@
         <v>79</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>7</v>
@@ -1926,7 +1926,7 @@
         <v>79</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>7</v>
@@ -2276,7 +2276,7 @@
         <v>124</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C96" s="7" t="s">
         <v>125</v>
@@ -2318,7 +2318,7 @@
         <v>129</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C99" s="7" t="s">
         <v>111</v>
@@ -2332,7 +2332,7 @@
         <v>129</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C100" s="7" t="s">
         <v>111</v>
@@ -2346,7 +2346,7 @@
         <v>129</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C101" s="7" t="s">
         <v>130</v>
@@ -2360,7 +2360,7 @@
         <v>129</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C102" s="7" t="s">
         <v>131</v>
@@ -2374,7 +2374,7 @@
         <v>129</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C103" s="7" t="s">
         <v>65</v>
@@ -2472,7 +2472,7 @@
         <v>141</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C110" s="7" t="s">
         <v>37</v>
@@ -2486,13 +2486,13 @@
         <v>141</v>
       </c>
       <c r="B111" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C111" s="7" t="s">
         <v>60</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -2500,10 +2500,10 @@
         <v>141</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2514,10 +2514,10 @@
         <v>141</v>
       </c>
       <c r="B113" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2528,7 +2528,7 @@
         <v>141</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C114" s="7" t="s">
         <v>34</v>
@@ -2542,7 +2542,7 @@
         <v>141</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C115" s="7" t="s">
         <v>37</v>
@@ -2556,7 +2556,7 @@
         <v>141</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C116" s="7" t="s">
         <v>7</v>
@@ -2570,13 +2570,13 @@
         <v>141</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C117" s="7" t="s">
         <v>42</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
@@ -2584,10 +2584,10 @@
         <v>141</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>48</v>
@@ -2595,27 +2595,27 @@
     </row>
     <row r="119" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C119" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B119" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="C119" s="7" t="s">
+      <c r="D119" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>4</v>
@@ -2623,13 +2623,13 @@
     </row>
     <row r="121" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B121" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C121" s="7" t="s">
         <v>152</v>
-      </c>
-      <c r="C121" s="7" t="s">
-        <v>153</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>48</v>
@@ -2637,10 +2637,10 @@
     </row>
     <row r="122" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C122" s="7" t="s">
         <v>37</v>
@@ -2651,10 +2651,10 @@
     </row>
     <row r="123" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123" s="7" t="s">
         <v>154</v>
-      </c>
-      <c r="B123" s="7" t="s">
-        <v>155</v>
       </c>
       <c r="C123" s="7" t="s">
         <v>118</v>
@@ -2665,13 +2665,13 @@
     </row>
     <row r="124" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B124" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B124" s="7" t="s">
+      <c r="C124" s="7" t="s">
         <v>155</v>
-      </c>
-      <c r="C124" s="7" t="s">
-        <v>156</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>119</v>
@@ -2679,13 +2679,13 @@
     </row>
     <row r="125" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B125" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B125" s="7" t="s">
+      <c r="C125" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="C125" s="7" t="s">
-        <v>159</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>119</v>
@@ -2693,10 +2693,10 @@
     </row>
     <row r="126" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B126" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="B126" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="C126" s="7" t="s">
         <v>103</v>
@@ -2707,10 +2707,10 @@
     </row>
     <row r="127" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B127" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="B127" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="C127" s="7" t="s">
         <v>135</v>
@@ -2721,13 +2721,13 @@
     </row>
     <row r="128" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B128" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B128" s="7" t="s">
-        <v>158</v>
-      </c>
       <c r="C128" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>4</v>
@@ -2735,24 +2735,24 @@
     </row>
     <row r="129" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>161</v>
+        <v>195</v>
       </c>
       <c r="C129" s="7" t="s">
         <v>133</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>161</v>
+        <v>195</v>
       </c>
       <c r="C130" s="7" t="s">
         <v>7</v>
@@ -2763,10 +2763,10 @@
     </row>
     <row r="131" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B131" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C131" s="7" t="s">
         <v>121</v>
@@ -2777,10 +2777,10 @@
     </row>
     <row r="132" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B132" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C132" s="7" t="s">
         <v>82</v>
@@ -2791,13 +2791,13 @@
     </row>
     <row r="133" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B133" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C133" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>68</v>
@@ -2805,10 +2805,10 @@
     </row>
     <row r="134" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C134" s="7" t="s">
         <v>135</v>
@@ -2819,10 +2819,10 @@
     </row>
     <row r="135" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C135" s="7" t="s">
         <v>103</v>
@@ -2833,13 +2833,13 @@
     </row>
     <row r="136" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B136" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B136" s="7" t="s">
-        <v>169</v>
-      </c>
       <c r="C136" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>68</v>
@@ -2847,13 +2847,13 @@
     </row>
     <row r="137" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B137" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C137" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>4</v>
@@ -2861,10 +2861,10 @@
     </row>
     <row r="138" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C138" s="7" t="s">
         <v>77</v>
@@ -2875,10 +2875,10 @@
     </row>
     <row r="139" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B139" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C139" s="7" t="s">
         <v>139</v>
@@ -2889,10 +2889,10 @@
     </row>
     <row r="140" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B140" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C140" s="7" t="s">
         <v>138</v>
@@ -2903,30 +2903,30 @@
     </row>
     <row r="141" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="C141" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B141" s="7" t="s">
+      <c r="D141" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="C141" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B142" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C142" s="7" t="s">
         <v>131</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>